<commit_message>
fix: retrain all models with properly scaled consumption data
- Consumption in tax_prepared_data.xlsx was measured in Actual PKR (e.g., ~ Trillion), whereas all other columns (GDP, GST, etc.) were in PKR Millions (e.g.,  Million).
- This massive scale discrepancy caused model coefficients on log_consumption to become unstable and create explosive forecasts (e.g., ARIMAX projecting 1.8 trillion PKR).
- The user divided consumption by 1,000,000.
- Re-ran Macro_Tax_Forecasting_Diag/train_prfs_ii.py to update tax_models_bundle.pkl and tax_models_meta.json.
- Model coefficients and residuals are now mathematically sound and correctly scaled to match the rest of the dataset.
</commit_message>
<xml_diff>
--- a/PRFS_II/tax_prepared_data.xlsx
+++ b/PRFS_II/tax_prepared_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\Downloads\Pakistan_Macro_Tax_Forecast\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\Downloads\Pakistan_Income_Tax_Slabs_app\PRFS_II\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D85DBC2F-B098-4E6F-B886-481485069A22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40697EAC-7DE1-4960-9831-EA43D9B5383B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9075" yWindow="525" windowWidth="9202" windowHeight="9878" xr2:uid="{ECD6AF0D-AEAE-44BC-8544-4540CC87867B}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10276" xr2:uid="{ECD6AF0D-AEAE-44BC-8544-4540CC87867B}"/>
   </bookViews>
   <sheets>
     <sheet name="tax_prepared_data" sheetId="1" r:id="rId1"/>
@@ -2251,6 +2251,7 @@
   <cols>
     <col min="2" max="2" width="17.19921875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15.59765625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.1328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:34" x14ac:dyDescent="0.45">
@@ -2395,7 +2396,7 @@
         <v>34</v>
       </c>
       <c r="M2">
-        <v>1570000000000</v>
+        <v>1570000</v>
       </c>
       <c r="N2">
         <v>0</v>
@@ -2496,7 +2497,7 @@
         <v>47</v>
       </c>
       <c r="M3">
-        <v>1810000000000</v>
+        <v>1810000</v>
       </c>
       <c r="N3">
         <v>0</v>
@@ -2600,7 +2601,7 @@
         <v>59</v>
       </c>
       <c r="M4">
-        <v>2110000000000</v>
+        <v>2110000</v>
       </c>
       <c r="N4">
         <v>0</v>
@@ -2704,7 +2705,7 @@
         <v>72</v>
       </c>
       <c r="M5">
-        <v>2230000000000</v>
+        <v>2230000</v>
       </c>
       <c r="N5">
         <v>0</v>
@@ -2808,7 +2809,7 @@
         <v>84</v>
       </c>
       <c r="M6">
-        <v>2530000000000</v>
+        <v>2530000</v>
       </c>
       <c r="N6">
         <v>0</v>
@@ -2912,7 +2913,7 @@
         <v>4.3605024175000002</v>
       </c>
       <c r="M7">
-        <v>4420000000000</v>
+        <v>4420000</v>
       </c>
       <c r="N7">
         <v>0</v>
@@ -3016,7 +3017,7 @@
         <v>112</v>
       </c>
       <c r="M8">
-        <v>4880000000000</v>
+        <v>4880000</v>
       </c>
       <c r="N8">
         <v>0</v>
@@ -3120,7 +3121,7 @@
         <v>128</v>
       </c>
       <c r="M9">
-        <v>5160000000000</v>
+        <v>5160000</v>
       </c>
       <c r="N9">
         <v>0</v>
@@ -3221,7 +3222,7 @@
         <v>144</v>
       </c>
       <c r="M10">
-        <v>5590000000000</v>
+        <v>5590000</v>
       </c>
       <c r="N10">
         <v>0</v>
@@ -3322,7 +3323,7 @@
         <v>159</v>
       </c>
       <c r="M11">
-        <v>6570000000000</v>
+        <v>6570000</v>
       </c>
       <c r="N11">
         <v>0</v>
@@ -3426,7 +3427,7 @@
         <v>9.0811006644999992</v>
       </c>
       <c r="M12">
-        <v>7680000000000</v>
+        <v>7680000</v>
       </c>
       <c r="N12">
         <v>0</v>
@@ -3530,7 +3531,7 @@
         <v>7.9168405100000001</v>
       </c>
       <c r="M13">
-        <v>8690000000000</v>
+        <v>8690000</v>
       </c>
       <c r="N13">
         <v>0</v>
@@ -3634,7 +3635,7 @@
         <v>202</v>
       </c>
       <c r="M14">
-        <v>10000000000000</v>
+        <v>10000000</v>
       </c>
       <c r="N14">
         <v>0</v>
@@ -3738,7 +3739,7 @@
         <v>218</v>
       </c>
       <c r="M15">
-        <v>11700000000000</v>
+        <v>11700000</v>
       </c>
       <c r="N15">
         <v>0</v>
@@ -3842,7 +3843,7 @@
         <v>234</v>
       </c>
       <c r="M16">
-        <v>13400000000000</v>
+        <v>13400000</v>
       </c>
       <c r="N16">
         <v>0</v>
@@ -3946,7 +3947,7 @@
         <v>249</v>
       </c>
       <c r="M17">
-        <v>15000000000000</v>
+        <v>15000000</v>
       </c>
       <c r="N17">
         <v>0</v>
@@ -4050,7 +4051,7 @@
         <v>265</v>
       </c>
       <c r="M18">
-        <v>17900000000000</v>
+        <v>17900000</v>
       </c>
       <c r="N18">
         <v>0</v>
@@ -4154,7 +4155,7 @@
         <v>281</v>
       </c>
       <c r="M19">
-        <v>20600000000000</v>
+        <v>20600000</v>
       </c>
       <c r="N19">
         <v>0</v>
@@ -4258,7 +4259,7 @@
         <v>295</v>
       </c>
       <c r="M20">
-        <v>22900000000000</v>
+        <v>22900000</v>
       </c>
       <c r="N20">
         <v>0</v>
@@ -4362,7 +4363,7 @@
         <v>311</v>
       </c>
       <c r="M21">
-        <v>25800000000000</v>
+        <v>25800000</v>
       </c>
       <c r="N21">
         <v>0</v>
@@ -4466,7 +4467,7 @@
         <v>323</v>
       </c>
       <c r="M22">
-        <v>27700000000000</v>
+        <v>27700000</v>
       </c>
       <c r="N22">
         <v>0</v>
@@ -4570,7 +4571,7 @@
         <v>336</v>
       </c>
       <c r="M23">
-        <v>29900000000000</v>
+        <v>29900000</v>
       </c>
       <c r="N23">
         <v>0</v>
@@ -4671,7 +4672,7 @@
         <v>5.3250000000000002</v>
       </c>
       <c r="M24">
-        <v>33000000000000</v>
+        <v>33000000</v>
       </c>
       <c r="N24">
         <v>0</v>
@@ -4775,7 +4776,7 @@
         <v>360</v>
       </c>
       <c r="M25">
-        <v>36600000000000</v>
+        <v>36600000</v>
       </c>
       <c r="N25">
         <v>1</v>
@@ -4879,7 +4880,7 @@
         <v>371</v>
       </c>
       <c r="M26">
-        <v>41400000000000</v>
+        <v>41400000</v>
       </c>
       <c r="N26">
         <v>1</v>
@@ -4983,7 +4984,7 @@
         <v>11.327020649750001</v>
       </c>
       <c r="M27">
-        <v>44400000000000</v>
+        <v>44400000</v>
       </c>
       <c r="N27">
         <v>0</v>
@@ -5087,7 +5088,7 @@
         <v>395</v>
       </c>
       <c r="M28">
-        <v>52700000000000</v>
+        <v>52700000</v>
       </c>
       <c r="N28">
         <v>0</v>
@@ -5191,7 +5192,7 @@
         <v>408</v>
       </c>
       <c r="M29">
-        <v>64300000000000</v>
+        <v>64300000</v>
       </c>
       <c r="N29">
         <v>0</v>
@@ -5295,7 +5296,7 @@
         <v>30.925000000000001</v>
       </c>
       <c r="M30">
-        <v>78200000000000</v>
+        <v>78200000</v>
       </c>
       <c r="N30">
         <v>0</v>
@@ -5399,7 +5400,7 @@
         <v>432</v>
       </c>
       <c r="M31">
-        <v>98500000000000</v>
+        <v>98500000</v>
       </c>
       <c r="N31">
         <v>0</v>

</xml_diff>